<commit_message>
Use agent and policy from the remastered branch for testing. Still doesn't work.
</commit_message>
<xml_diff>
--- a/applications/tracking_disturbance_3species_reinforce/Discover_Molecular_Integrators_REINFORCE.xlsx
+++ b/applications/tracking_disturbance_3species_reinforce/Discover_Molecular_Integrators_REINFORCE.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH27"/>
+  <dimension ref="A1:AW27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,6 +587,81 @@
           <t>2025-09-15 09:30:03</t>
         </is>
       </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>2025-09-15 09:59:44</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>2025-09-15 10:11:40</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>2025-09-15 10:15:06</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>2025-09-15 10:15:43</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>2025-09-15 10:19:03</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>2025-09-15 10:32:35</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>2025-09-15 10:33:05</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>2025-09-15 10:33:40</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>2025-09-15 10:37:47</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>2025-09-15 13:36:16</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>2025-09-15 13:36:30</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>2025-09-15 13:37:14</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>2025-09-15 13:40:00</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>2025-09-15 13:42:12</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>2025-09-15 13:49:14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -759,6 +834,81 @@
           <t>https://www.comet.com/maurice-filo/molecular-integrators/ea4d8f4f3b0e44399119ca3814b678d7</t>
         </is>
       </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/4b708de3411745469c997df7afaed569</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/e88215bdd548403091bdfd5a8bc6194d</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/da4388ed83e1412fbd26fbafbf7945b3</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/c84577775ea444c787dc5e7a2dc651fd</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/b5323f913ba24f2297f27bd1798475b7</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/65e71c3577c44bbd8ae9342e6556ac17</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/bdc5effe74954cec9eb3cda52cf6a85f</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/c5dc6a82f53642118842a581333f9fbd</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/78cd3977fcba4220a16f5ffbd97b7edd</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/9d6d02be275f4eb0840e2d059e7398e4</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/1ec320ae5e1a488c8eb2c0e47b953ce5</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/d0cdc579031f4a0185b0cdfe6ac291e7</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/e85fc51a0ccf4f5a981d250ade24ebc4</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/33efb0ae3b754af68a0af369020e51b0</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/e64f49daac3a4bc28d80af1d4c31a23a</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -865,6 +1015,51 @@
       <c r="AH3" t="n">
         <v>5</v>
       </c>
+      <c r="AI3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -971,6 +1166,51 @@
       <c r="AH4" t="n">
         <v>3</v>
       </c>
+      <c r="AI4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1077,6 +1317,51 @@
       <c r="AH5" t="n">
         <v>2</v>
       </c>
+      <c r="AI5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1183,6 +1468,51 @@
       <c r="AH6" t="n">
         <v>1280</v>
       </c>
+      <c r="AI6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>1280</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1289,6 +1619,51 @@
       <c r="AH7" t="b">
         <v>0</v>
       </c>
+      <c r="AI7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AU7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1395,6 +1770,51 @@
       <c r="AH8" t="n">
         <v>0.0001</v>
       </c>
+      <c r="AI8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1501,6 +1921,51 @@
       <c r="AH9" t="n">
         <v>500</v>
       </c>
+      <c r="AI9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>500</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1607,6 +2072,51 @@
       <c r="AH10" t="n">
         <v>5</v>
       </c>
+      <c r="AI10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1713,6 +2223,51 @@
       <c r="AH11" t="n">
         <v>1024</v>
       </c>
+      <c r="AI11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1819,6 +2374,51 @@
       <c r="AH12" t="n">
         <v>10240</v>
       </c>
+      <c r="AI12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>10240</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>10240</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1925,6 +2525,51 @@
       <c r="AH13" t="n">
         <v>128</v>
       </c>
+      <c r="AI13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>128</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2031,6 +2676,51 @@
       <c r="AH14" t="n">
         <v>50</v>
       </c>
+      <c r="AI14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2137,6 +2827,51 @@
       <c r="AH15" t="n">
         <v>0.75</v>
       </c>
+      <c r="AI15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2243,6 +2978,51 @@
       <c r="AH16" t="n">
         <v>5</v>
       </c>
+      <c r="AI16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2349,6 +3129,51 @@
       <c r="AH17" t="n">
         <v>50</v>
       </c>
+      <c r="AI17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>50</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2455,6 +3280,51 @@
       <c r="AH18" t="n">
         <v>0.95</v>
       </c>
+      <c r="AI18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AS18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>0.95</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2561,6 +3431,51 @@
       <c r="AH19" t="n">
         <v>0</v>
       </c>
+      <c r="AI19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2667,6 +3582,51 @@
       <c r="AH20" t="n">
         <v>1</v>
       </c>
+      <c r="AI20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2773,6 +3733,51 @@
       <c r="AH21" t="n">
         <v>20</v>
       </c>
+      <c r="AI21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AP21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AR21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AS21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AV21" t="n">
+        <v>20</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2879,6 +3884,51 @@
       <c r="AH22" t="n">
         <v>1</v>
       </c>
+      <c r="AI22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2985,6 +4035,51 @@
       <c r="AH23" t="n">
         <v>10</v>
       </c>
+      <c r="AI23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AO23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AP23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AR23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AS23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>10</v>
+      </c>
+      <c r="AW23" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3091,6 +4186,51 @@
       <c r="AH24" t="n">
         <v>200</v>
       </c>
+      <c r="AI24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>200</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3197,6 +4337,51 @@
       <c r="AH25" t="n">
         <v>1000</v>
       </c>
+      <c r="AI25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AV25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AW25" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3303,6 +4488,51 @@
       <c r="AH26" t="n">
         <v>1</v>
       </c>
+      <c r="AI26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3407,6 +4637,51 @@
         <v>9</v>
       </c>
       <c r="AH27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AW27" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added compile() to add_reaction() in IOCRN.
</commit_message>
<xml_diff>
--- a/applications/tracking_disturbance_3species_reinforce/Discover_Molecular_Integrators_REINFORCE.xlsx
+++ b/applications/tracking_disturbance_3species_reinforce/Discover_Molecular_Integrators_REINFORCE.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW27"/>
+  <dimension ref="A1:AX27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -662,6 +662,11 @@
           <t>2025-09-15 13:49:14</t>
         </is>
       </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>2025-09-15 19:28:35</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -909,6 +914,11 @@
           <t>https://www.comet.com/maurice-filo/molecular-integrators/e64f49daac3a4bc28d80af1d4c31a23a</t>
         </is>
       </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/3072284f12aa49588adeabed17667611</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1060,6 +1070,9 @@
       <c r="AW3" t="n">
         <v>5</v>
       </c>
+      <c r="AX3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1211,6 +1224,9 @@
       <c r="AW4" t="n">
         <v>3</v>
       </c>
+      <c r="AX4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1362,6 +1378,9 @@
       <c r="AW5" t="n">
         <v>2</v>
       </c>
+      <c r="AX5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1513,6 +1532,9 @@
       <c r="AW6" t="n">
         <v>1280</v>
       </c>
+      <c r="AX6" t="n">
+        <v>1280</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1664,6 +1686,9 @@
       <c r="AW7" t="b">
         <v>0</v>
       </c>
+      <c r="AX7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1815,6 +1840,9 @@
       <c r="AW8" t="n">
         <v>0.0001</v>
       </c>
+      <c r="AX8" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1966,6 +1994,9 @@
       <c r="AW9" t="n">
         <v>500</v>
       </c>
+      <c r="AX9" t="n">
+        <v>500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2117,6 +2148,9 @@
       <c r="AW10" t="n">
         <v>5</v>
       </c>
+      <c r="AX10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2268,6 +2302,9 @@
       <c r="AW11" t="n">
         <v>1024</v>
       </c>
+      <c r="AX11" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2419,6 +2456,9 @@
       <c r="AW12" t="n">
         <v>10240</v>
       </c>
+      <c r="AX12" t="n">
+        <v>10240</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2570,6 +2610,9 @@
       <c r="AW13" t="n">
         <v>128</v>
       </c>
+      <c r="AX13" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2721,6 +2764,9 @@
       <c r="AW14" t="n">
         <v>50</v>
       </c>
+      <c r="AX14" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2872,6 +2918,9 @@
       <c r="AW15" t="n">
         <v>0.75</v>
       </c>
+      <c r="AX15" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3023,6 +3072,9 @@
       <c r="AW16" t="n">
         <v>5</v>
       </c>
+      <c r="AX16" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3174,6 +3226,9 @@
       <c r="AW17" t="n">
         <v>50</v>
       </c>
+      <c r="AX17" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3325,6 +3380,9 @@
       <c r="AW18" t="n">
         <v>0.95</v>
       </c>
+      <c r="AX18" t="n">
+        <v>0.95</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3476,6 +3534,9 @@
       <c r="AW19" t="n">
         <v>0</v>
       </c>
+      <c r="AX19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3627,6 +3688,9 @@
       <c r="AW20" t="n">
         <v>1</v>
       </c>
+      <c r="AX20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3778,6 +3842,9 @@
       <c r="AW21" t="n">
         <v>20</v>
       </c>
+      <c r="AX21" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3929,6 +3996,9 @@
       <c r="AW22" t="n">
         <v>1</v>
       </c>
+      <c r="AX22" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4080,6 +4150,9 @@
       <c r="AW23" t="n">
         <v>10</v>
       </c>
+      <c r="AX23" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4231,6 +4304,9 @@
       <c r="AW24" t="n">
         <v>200</v>
       </c>
+      <c r="AX24" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4382,6 +4458,9 @@
       <c r="AW25" t="n">
         <v>1000</v>
       </c>
+      <c r="AX25" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4533,6 +4612,9 @@
       <c r="AW26" t="n">
         <v>1</v>
       </c>
+      <c r="AX26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4682,6 +4764,9 @@
         <v>9</v>
       </c>
       <c r="AW27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AX27" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>